<commit_message>
updating module catalogue with new ID5059 timetable
</commit_message>
<xml_diff>
--- a/src/advising/Module_catalogue.xlsx
+++ b/src/advising/Module_catalogue.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofstandrews907-my.sharepoint.com/personal/dwrj1_st-andrews_ac_uk/Documents/DoT/Advising/Advising-tool/StA_Advising/src/advising/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk263/projects/StA_Advising/src/advising/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{84145898-1FC4-A746-8358-CC0400B61A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABD784D5-B4AC-7642-BF28-8CDF43B432A5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21B7744-B08E-C14A-A216-EAEA90B7EE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19820" xr2:uid="{4F9A127D-94E5-E147-ADFA-9B9D4F5F7BAB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="297">
   <si>
     <t>Module code</t>
   </si>
@@ -924,6 +924,9 @@
   </si>
   <si>
     <t>2026/2027</t>
+  </si>
+  <si>
+    <t>5pm Mon, 5pm Tue</t>
   </si>
 </sst>
 </file>
@@ -1409,7 +1412,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>296</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Further changes ahead of AY26_27, MT5855/56 timetable change and MT5590 (S2) only.
</commit_message>
<xml_diff>
--- a/src/advising/Module_catalogue.xlsx
+++ b/src/advising/Module_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofstandrews907-my.sharepoint.com/personal/dwrj1_st-andrews_ac_uk/Documents/DoT/Advising/Advising-tool/StA_Advising/src/advising/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{512B0E99-D0D4-904E-9A76-C0B28B78645E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E109DBEB-F648-DD4A-B4B8-63BF3585FFA2}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{512B0E99-D0D4-904E-9A76-C0B28B78645E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A35AD11E-3F4C-3242-9ADE-F9D7EBF4B636}"/>
   <bookViews>
     <workbookView xWindow="1760" yWindow="800" windowWidth="29400" windowHeight="17160" xr2:uid="{4F9A127D-94E5-E147-ADFA-9B9D4F5F7BAB}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$104</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="323">
   <si>
     <t>Module code</t>
   </si>
@@ -1390,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692125B0-B9FD-1C45-BA4C-1792B9B50D49}">
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.83203125" style="1" customWidth="1"/>
@@ -1465,7 +1465,7 @@
         <v>296</v>
       </c>
       <c r="J2" s="1" t="str">
-        <f>IF(VALUE(LEFT(C2,4))&gt;2050,"Temp withdrawal",IF(F2="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C2,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" ref="J2:J33" si="0">IF(VALUE(LEFT(C2,4))&gt;2050,"Temp withdrawal",IF(F2="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C2,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
         <v>296</v>
       </c>
       <c r="J3" s="1" t="str">
-        <f>IF(VALUE(LEFT(C3,4))&gt;2050,"Temp withdrawal",IF(F3="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C3,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
         <v>296</v>
       </c>
       <c r="J4" s="1" t="str">
-        <f>IF(VALUE(LEFT(C4,4))&gt;2050,"Temp withdrawal",IF(F4="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C4,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
         <v>299</v>
       </c>
       <c r="J5" s="1" t="str">
-        <f>IF(VALUE(LEFT(C5,4))&gt;2050,"Temp withdrawal",IF(F5="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C5,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
         <v>299</v>
       </c>
       <c r="J6" s="1" t="str">
-        <f>IF(VALUE(LEFT(C6,4))&gt;2050,"Temp withdrawal",IF(F6="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C6,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
         <v>299</v>
       </c>
       <c r="J7" s="1" t="str">
-        <f>IF(VALUE(LEFT(C7,4))&gt;2050,"Temp withdrawal",IF(F7="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C7,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
         <v>299</v>
       </c>
       <c r="J8" s="1" t="str">
-        <f>IF(VALUE(LEFT(C8,4))&gt;2050,"Temp withdrawal",IF(F8="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C8,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
         <v>296</v>
       </c>
       <c r="J9" s="1" t="str">
-        <f>IF(VALUE(LEFT(C9,4))&gt;2050,"Temp withdrawal",IF(F9="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C9,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
         <v>299</v>
       </c>
       <c r="J10" s="1" t="str">
-        <f>IF(VALUE(LEFT(C10,4))&gt;2050,"Temp withdrawal",IF(F10="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C10,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
         <v>299</v>
       </c>
       <c r="J11" s="1" t="str">
-        <f>IF(VALUE(LEFT(C11,4))&gt;2050,"Temp withdrawal",IF(F11="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C11,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
         <v>301</v>
       </c>
       <c r="J12" s="1" t="str">
-        <f>IF(VALUE(LEFT(C12,4))&gt;2050,"Temp withdrawal",IF(F12="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C12,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
         <v>302</v>
       </c>
       <c r="J13" s="1" t="str">
-        <f>IF(VALUE(LEFT(C13,4))&gt;2050,"Temp withdrawal",IF(F13="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C13,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
         <v>302</v>
       </c>
       <c r="J14" s="1" t="str">
-        <f>IF(VALUE(LEFT(C14,4))&gt;2050,"Temp withdrawal",IF(F14="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C14,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
         <v>303</v>
       </c>
       <c r="J15" s="1" t="str">
-        <f>IF(VALUE(LEFT(C15,4))&gt;2050,"Temp withdrawal",IF(F15="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C15,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
         <v>301</v>
       </c>
       <c r="J16" s="1" t="str">
-        <f>IF(VALUE(LEFT(C16,4))&gt;2050,"Temp withdrawal",IF(F16="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C16,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
         <v>302</v>
       </c>
       <c r="J17" s="1" t="str">
-        <f>IF(VALUE(LEFT(C17,4))&gt;2050,"Temp withdrawal",IF(F17="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C17,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
         <v>302</v>
       </c>
       <c r="J18" s="1" t="str">
-        <f>IF(VALUE(LEFT(C18,4))&gt;2050,"Temp withdrawal",IF(F18="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C18,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
         <v>296</v>
       </c>
       <c r="J19" s="1" t="str">
-        <f>IF(VALUE(LEFT(C19,4))&gt;2050,"Temp withdrawal",IF(F19="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C19,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
         <v>304</v>
       </c>
       <c r="J20" s="1" t="str">
-        <f>IF(VALUE(LEFT(C20,4))&gt;2050,"Temp withdrawal",IF(F20="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C20,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Temp withdrawal</v>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
         <v>301</v>
       </c>
       <c r="J21" s="1" t="str">
-        <f>IF(VALUE(LEFT(C21,4))&gt;2050,"Temp withdrawal",IF(F21="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C21,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
         <v>301</v>
       </c>
       <c r="J22" s="1" t="str">
-        <f>IF(VALUE(LEFT(C22,4))&gt;2050,"Temp withdrawal",IF(F22="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C22,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
         <v>299</v>
       </c>
       <c r="J23" s="1" t="str">
-        <f>IF(VALUE(LEFT(C23,4))&gt;2050,"Temp withdrawal",IF(F23="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C23,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
         <v>302</v>
       </c>
       <c r="J24" s="1" t="str">
-        <f>IF(VALUE(LEFT(C24,4))&gt;2050,"Temp withdrawal",IF(F24="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C24,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
         <v>301</v>
       </c>
       <c r="J25" s="1" t="str">
-        <f>IF(VALUE(LEFT(C25,4))&gt;2050,"Temp withdrawal",IF(F25="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C25,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
         <v>302</v>
       </c>
       <c r="J26" s="1" t="str">
-        <f>IF(VALUE(LEFT(C26,4))&gt;2050,"Temp withdrawal",IF(F26="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C26,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2223,7 +2223,7 @@
         <v>296</v>
       </c>
       <c r="J27" s="1" t="str">
-        <f>IF(VALUE(LEFT(C27,4))&gt;2050,"Temp withdrawal",IF(F27="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C27,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
         <v>296</v>
       </c>
       <c r="J28" s="1" t="str">
-        <f>IF(VALUE(LEFT(C28,4))&gt;2050,"Temp withdrawal",IF(F28="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C28,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
         <v>313</v>
       </c>
       <c r="J29" s="1" t="str">
-        <f>IF(VALUE(LEFT(C29,4))&gt;2050,"Temp withdrawal",IF(F29="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C29,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
         <v>301</v>
       </c>
       <c r="J30" s="1" t="str">
-        <f>IF(VALUE(LEFT(C30,4))&gt;2050,"Temp withdrawal",IF(F30="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C30,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
         <v>301</v>
       </c>
       <c r="J31" s="1" t="str">
-        <f>IF(VALUE(LEFT(C31,4))&gt;2050,"Temp withdrawal",IF(F31="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C31,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
         <v>302</v>
       </c>
       <c r="J32" s="1" t="str">
-        <f>IF(VALUE(LEFT(C32,4))&gt;2050,"Temp withdrawal",IF(F32="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C32,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
         <v>302</v>
       </c>
       <c r="J33" s="1" t="str">
-        <f>IF(VALUE(LEFT(C33,4))&gt;2050,"Temp withdrawal",IF(F33="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C33,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="0"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2433,7 +2433,7 @@
         <v>296</v>
       </c>
       <c r="J34" s="1" t="str">
-        <f>IF(VALUE(LEFT(C34,4))&gt;2050,"Temp withdrawal",IF(F34="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C34,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" ref="J34:J65" si="1">IF(VALUE(LEFT(C34,4))&gt;2050,"Temp withdrawal",IF(F34="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C34,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
         <v>304</v>
       </c>
       <c r="J35" s="1" t="str">
-        <f>IF(VALUE(LEFT(C35,4))&gt;2050,"Temp withdrawal",IF(F35="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C35,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
         <v>302</v>
       </c>
       <c r="J36" s="1" t="str">
-        <f>IF(VALUE(LEFT(C36,4))&gt;2050,"Temp withdrawal",IF(F36="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C36,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2529,7 +2529,7 @@
         <v>302</v>
       </c>
       <c r="J37" s="1" t="str">
-        <f>IF(VALUE(LEFT(C37,4))&gt;2050,"Temp withdrawal",IF(F37="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C37,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
         <v>302</v>
       </c>
       <c r="J38" s="1" t="str">
-        <f>IF(VALUE(LEFT(C38,4))&gt;2050,"Temp withdrawal",IF(F38="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C38,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
         <v>302</v>
       </c>
       <c r="J39" s="1" t="str">
-        <f>IF(VALUE(LEFT(C39,4))&gt;2050,"Temp withdrawal",IF(F39="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C39,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
         <v>302</v>
       </c>
       <c r="J40" s="1" t="str">
-        <f>IF(VALUE(LEFT(C40,4))&gt;2050,"Temp withdrawal",IF(F40="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C40,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
         <v>301</v>
       </c>
       <c r="J41" s="1" t="str">
-        <f>IF(VALUE(LEFT(C41,4))&gt;2050,"Temp withdrawal",IF(F41="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C41,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
         <v>301</v>
       </c>
       <c r="J42" s="1" t="str">
-        <f>IF(VALUE(LEFT(C42,4))&gt;2050,"Temp withdrawal",IF(F42="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C42,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
         <v>301</v>
       </c>
       <c r="J43" s="1" t="str">
-        <f>IF(VALUE(LEFT(C43,4))&gt;2050,"Temp withdrawal",IF(F43="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C43,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
         <v>301</v>
       </c>
       <c r="J44" s="1" t="str">
-        <f>IF(VALUE(LEFT(C44,4))&gt;2050,"Temp withdrawal",IF(F44="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C44,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
         <v>301</v>
       </c>
       <c r="J45" s="1" t="str">
-        <f>IF(VALUE(LEFT(C45,4))&gt;2050,"Temp withdrawal",IF(F45="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C45,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2802,7 +2802,7 @@
         <v>301</v>
       </c>
       <c r="J46" s="1" t="str">
-        <f>IF(VALUE(LEFT(C46,4))&gt;2050,"Temp withdrawal",IF(F46="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C46,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
         <v>301</v>
       </c>
       <c r="J47" s="1" t="str">
-        <f>IF(VALUE(LEFT(C47,4))&gt;2050,"Temp withdrawal",IF(F47="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C47,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
         <v>296</v>
       </c>
       <c r="J48" s="1" t="str">
-        <f>IF(VALUE(LEFT(C48,4))&gt;2050,"Temp withdrawal",IF(F48="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C48,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
         <v>296</v>
       </c>
       <c r="J49" s="1" t="str">
-        <f>IF(VALUE(LEFT(C49,4))&gt;2050,"Temp withdrawal",IF(F49="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C49,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
         <v>296</v>
       </c>
       <c r="J50" s="1" t="str">
-        <f>IF(VALUE(LEFT(C50,4))&gt;2050,"Temp withdrawal",IF(F50="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C50,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Temp withdrawal</v>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
         <v>296</v>
       </c>
       <c r="J51" s="1" t="str">
-        <f>IF(VALUE(LEFT(C51,4))&gt;2050,"Temp withdrawal",IF(F51="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C51,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -2985,7 +2985,7 @@
         <v>296</v>
       </c>
       <c r="J52" s="1" t="str">
-        <f>IF(VALUE(LEFT(C52,4))&gt;2050,"Temp withdrawal",IF(F52="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C52,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Temp withdrawal</v>
       </c>
     </row>
@@ -3015,7 +3015,7 @@
         <v>296</v>
       </c>
       <c r="J53" s="1" t="str">
-        <f>IF(VALUE(LEFT(C53,4))&gt;2050,"Temp withdrawal",IF(F53="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C53,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Temp withdrawal</v>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
         <v>302</v>
       </c>
       <c r="J54" s="1" t="str">
-        <f>IF(VALUE(LEFT(C54,4))&gt;2050,"Temp withdrawal",IF(F54="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C54,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
         <v>302</v>
       </c>
       <c r="J55" s="1" t="str">
-        <f>IF(VALUE(LEFT(C55,4))&gt;2050,"Temp withdrawal",IF(F55="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C55,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3108,7 +3108,7 @@
         <v>302</v>
       </c>
       <c r="J56" s="1" t="str">
-        <f>IF(VALUE(LEFT(C56,4))&gt;2050,"Temp withdrawal",IF(F56="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C56,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
         <v>302</v>
       </c>
       <c r="J57" s="1" t="str">
-        <f>IF(VALUE(LEFT(C57,4))&gt;2050,"Temp withdrawal",IF(F57="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C57,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
         <v>304</v>
       </c>
       <c r="J58" s="1" t="str">
-        <f>IF(VALUE(LEFT(C58,4))&gt;2050,"Temp withdrawal",IF(F58="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C58,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
         <v>296</v>
       </c>
       <c r="J59" s="1" t="str">
-        <f>IF(VALUE(LEFT(C59,4))&gt;2050,"Temp withdrawal",IF(F59="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C59,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
         <v>296</v>
       </c>
       <c r="J60" s="1" t="str">
-        <f>IF(VALUE(LEFT(C60,4))&gt;2050,"Temp withdrawal",IF(F60="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C60,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
         <v>314</v>
       </c>
       <c r="J61" s="1" t="str">
-        <f>IF(VALUE(LEFT(C61,4))&gt;2050,"Temp withdrawal",IF(F61="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C61,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
         <v>314</v>
       </c>
       <c r="J62" s="1" t="str">
-        <f>IF(VALUE(LEFT(C62,4))&gt;2050,"Temp withdrawal",IF(F62="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C62,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
         <v>296</v>
       </c>
       <c r="J63" s="1" t="str">
-        <f>IF(VALUE(LEFT(C63,4))&gt;2050,"Temp withdrawal",IF(F63="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C63,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
         <v>296</v>
       </c>
       <c r="J64" s="1" t="str">
-        <f>IF(VALUE(LEFT(C64,4))&gt;2050,"Temp withdrawal",IF(F64="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C64,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
         <v>296</v>
       </c>
       <c r="J65" s="1" t="str">
-        <f>IF(VALUE(LEFT(C65,4))&gt;2050,"Temp withdrawal",IF(F65="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C65,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="1"/>
         <v>Temp withdrawal</v>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
         <v>314</v>
       </c>
       <c r="J66" s="1" t="str">
-        <f>IF(VALUE(LEFT(C66,4))&gt;2050,"Temp withdrawal",IF(F66="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C66,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" ref="J66:J96" si="2">IF(VALUE(LEFT(C66,4))&gt;2050,"Temp withdrawal",IF(F66="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C66,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
         <v>314</v>
       </c>
       <c r="J67" s="1" t="str">
-        <f>IF(VALUE(LEFT(C67,4))&gt;2050,"Temp withdrawal",IF(F67="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C67,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
         <v>314</v>
       </c>
       <c r="J68" s="1" t="str">
-        <f>IF(VALUE(LEFT(C68,4))&gt;2050,"Temp withdrawal",IF(F68="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C68,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3474,7 +3474,7 @@
         <v>314</v>
       </c>
       <c r="J69" s="1" t="str">
-        <f>IF(VALUE(LEFT(C69,4))&gt;2050,"Temp withdrawal",IF(F69="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C69,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
         <v>314</v>
       </c>
       <c r="J70" s="1" t="str">
-        <f>IF(VALUE(LEFT(C70,4))&gt;2050,"Temp withdrawal",IF(F70="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C70,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
         <v>314</v>
       </c>
       <c r="J71" s="1" t="str">
-        <f>IF(VALUE(LEFT(C71,4))&gt;2050,"Temp withdrawal",IF(F71="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C71,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
         <v>10</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>13</v>
@@ -3548,104 +3548,110 @@
       <c r="G72" s="1" t="s">
         <v>147</v>
       </c>
+      <c r="H72" s="1" t="s">
+        <v>266</v>
+      </c>
       <c r="I72" s="1" t="s">
         <v>314</v>
       </c>
       <c r="J72" s="1" t="str">
-        <f>IF(VALUE(LEFT(C72,4))&gt;2050,"Temp withdrawal",IF(F72="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C72,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>147</v>
       </c>
       <c r="I73" s="1" t="s">
         <v>314</v>
       </c>
       <c r="J73" s="1" t="str">
-        <f>IF(VALUE(LEFT(C73,4))&gt;2050,"Temp withdrawal",IF(F73="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C73,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>146</v>
+        <v>15</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>13</v>
+        <v>80</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>314</v>
+        <v>296</v>
       </c>
       <c r="J74" s="1" t="str">
-        <f>IF(VALUE(LEFT(C74,4))&gt;2050,"Temp withdrawal",IF(F74="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C74,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Runs every year</v>
+        <f t="shared" si="2"/>
+        <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>128</v>
+        <v>10</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="I75" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J75" s="1" t="str">
-        <f>IF(VALUE(LEFT(C75,4))&gt;2050,"Temp withdrawal",IF(F75="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C75,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2026/27)</v>
+        <f t="shared" si="2"/>
+        <v>Runs every year</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>10</v>
@@ -3654,61 +3660,64 @@
         <v>15</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>179</v>
+        <v>124</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>182</v>
       </c>
       <c r="I76" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J76" s="1" t="str">
-        <f>IF(VALUE(LEFT(C76,4))&gt;2050,"Temp withdrawal",IF(F76="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C76,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>16</v>
+        <v>185</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>124</v>
+        <v>186</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="I77" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J77" s="1" t="str">
-        <f>IF(VALUE(LEFT(C77,4))&gt;2050,"Temp withdrawal",IF(F77="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C77,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>10</v>
@@ -3717,31 +3726,31 @@
         <v>11</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="I78" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J78" s="1" t="str">
-        <f>IF(VALUE(LEFT(C78,4))&gt;2050,"Temp withdrawal",IF(F78="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C78,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>10</v>
@@ -3750,7 +3759,7 @@
         <v>11</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>190</v>
+        <v>21</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>13</v>
@@ -3759,28 +3768,28 @@
         <v>191</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>192</v>
+        <v>74</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J79" s="1" t="str">
-        <f>IF(VALUE(LEFT(C79,4))&gt;2050,"Temp withdrawal",IF(F79="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C79,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>21</v>
@@ -3789,148 +3798,148 @@
         <v>13</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>74</v>
+        <v>198</v>
       </c>
       <c r="I80" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J80" s="1" t="str">
-        <f>IF(VALUE(LEFT(C80,4))&gt;2050,"Temp withdrawal",IF(F80="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C80,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>198</v>
+        <v>124</v>
       </c>
       <c r="I81" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J81" s="1" t="str">
-        <f>IF(VALUE(LEFT(C81,4))&gt;2050,"Temp withdrawal",IF(F81="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C81,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Runs every year</v>
+        <f t="shared" si="2"/>
+        <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>84</v>
+        <v>203</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>124</v>
+        <v>281</v>
       </c>
       <c r="I82" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J82" s="1" t="str">
-        <f>IF(VALUE(LEFT(C82,4))&gt;2050,"Temp withdrawal",IF(F82="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C82,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2027/28)</v>
+        <f t="shared" si="2"/>
+        <v>Runs every year</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>128</v>
+        <v>10</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>146</v>
+        <v>11</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>203</v>
+        <v>71</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>281</v>
+        <v>124</v>
       </c>
       <c r="I83" s="1" t="s">
         <v>296</v>
       </c>
       <c r="J83" s="1" t="str">
-        <f>IF(VALUE(LEFT(C83,4))&gt;2050,"Temp withdrawal",IF(F83="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C83,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>124</v>
+        <v>44</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>208</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="J84" s="1" t="str">
-        <f>IF(VALUE(LEFT(C84,4))&gt;2050,"Temp withdrawal",IF(F84="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C84,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>10</v>
@@ -3939,61 +3948,61 @@
         <v>15</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H85" s="1" t="s">
-        <v>208</v>
+        <v>68</v>
       </c>
       <c r="I85" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J85" s="1" t="str">
-        <f>IF(VALUE(LEFT(C85,4))&gt;2050,"Temp withdrawal",IF(F85="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C85,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>68</v>
+        <v>89</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>213</v>
       </c>
       <c r="I86" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J86" s="1" t="str">
-        <f>IF(VALUE(LEFT(C86,4))&gt;2050,"Temp withdrawal",IF(F86="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C86,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>10</v>
@@ -4002,31 +4011,31 @@
         <v>11</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I87" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J87" s="1" t="str">
-        <f>IF(VALUE(LEFT(C87,4))&gt;2050,"Temp withdrawal",IF(F87="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C87,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>10</v>
@@ -4035,37 +4044,37 @@
         <v>11</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="I88" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J88" s="1" t="str">
-        <f>IF(VALUE(LEFT(C88,4))&gt;2050,"Temp withdrawal",IF(F88="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C88,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>22</v>
@@ -4076,119 +4085,119 @@
       <c r="G89" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H89" s="1" t="s">
-        <v>219</v>
-      </c>
       <c r="I89" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J89" s="1" t="str">
-        <f>IF(VALUE(LEFT(C89,4))&gt;2050,"Temp withdrawal",IF(F89="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C89,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Runs every year</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>221</v>
+        <v>288</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>10</v>
+        <v>121</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>47</v>
+        <v>289</v>
       </c>
       <c r="I90" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J90" s="1" t="str">
-        <f>IF(VALUE(LEFT(C90,4))&gt;2050,"Temp withdrawal",IF(F90="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C90,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Runs every year</v>
+        <f t="shared" si="2"/>
+        <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>288</v>
+        <v>224</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>121</v>
+        <v>320</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>289</v>
+        <v>47</v>
       </c>
       <c r="I91" s="1" t="s">
         <v>302</v>
       </c>
       <c r="J91" s="1" t="str">
-        <f>IF(VALUE(LEFT(C91,4))&gt;2050,"Temp withdrawal",IF(F91="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C91,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2027/28)</v>
+        <f t="shared" si="2"/>
+        <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>320</v>
+        <v>70</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>47</v>
+        <v>227</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>228</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J92" s="1" t="str">
-        <f>IF(VALUE(LEFT(C92,4))&gt;2050,"Temp withdrawal",IF(F92="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C92,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2026/27)</v>
+        <f t="shared" si="2"/>
+        <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>70</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>12</v>
@@ -4197,121 +4206,121 @@
         <v>80</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="H93" s="1" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="I93" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J93" s="1" t="str">
-        <f>IF(VALUE(LEFT(C93,4))&gt;2050,"Temp withdrawal",IF(F93="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C93,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>70</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>12</v>
+        <v>234</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>231</v>
+        <v>235</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>236</v>
       </c>
       <c r="I94" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J94" s="1" t="str">
-        <f>IF(VALUE(LEFT(C94,4))&gt;2050,"Temp withdrawal",IF(F94="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C94,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>70</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>234</v>
+        <v>71</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>235</v>
+        <v>62</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="I95" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J95" s="1" t="str">
-        <f>IF(VALUE(LEFT(C95,4))&gt;2050,"Temp withdrawal",IF(F95="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C95,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="2"/>
         <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="G96" s="1" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="I96" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J96" s="1" t="str">
-        <f>IF(VALUE(LEFT(C96,4))&gt;2050,"Temp withdrawal",IF(F96="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C96,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2027/28)</v>
+        <f t="shared" si="2"/>
+        <v>Runs every year</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>10</v>
@@ -4320,130 +4329,127 @@
         <v>11</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H97" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I97" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J97" s="1" t="str">
-        <f>IF(VALUE(LEFT(C97,4))&gt;2050,"Temp withdrawal",IF(F97="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C97,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Runs every year</v>
+        <f t="shared" ref="J97:J106" si="3">IF(VALUE(LEFT(C97,4))&gt;2050,"Temp withdrawal",IF(F97="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C97,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>245</v>
+        <v>248</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>249</v>
       </c>
       <c r="I98" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J98" s="1" t="str">
-        <f>IF(VALUE(LEFT(C98,4))&gt;2050,"Temp withdrawal",IF(F98="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C98,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="3"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>10</v>
+        <v>286</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="H99" s="1" t="s">
-        <v>249</v>
+        <v>49</v>
       </c>
       <c r="I99" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J99" s="1" t="str">
-        <f>IF(VALUE(LEFT(C99,4))&gt;2050,"Temp withdrawal",IF(F99="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C99,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2026/27)</v>
+        <f t="shared" si="3"/>
+        <v>Temp withdrawal</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>286</v>
+        <v>128</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>49</v>
+        <v>254</v>
       </c>
       <c r="I100" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J100" s="1" t="str">
-        <f>IF(VALUE(LEFT(C100,4))&gt;2050,"Temp withdrawal",IF(F100="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C100,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Temp withdrawal</v>
+        <f t="shared" si="3"/>
+        <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>128</v>
+        <v>10</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>71</v>
@@ -4452,58 +4458,58 @@
         <v>80</v>
       </c>
       <c r="G101" s="1" t="s">
-        <v>254</v>
+        <v>257</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>258</v>
       </c>
       <c r="I101" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J101" s="1" t="str">
-        <f>IF(VALUE(LEFT(C101,4))&gt;2050,"Temp withdrawal",IF(F101="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C101,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="3"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A102" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>256</v>
+      <c r="A102" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>306</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>10</v>
+        <v>320</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>80</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="H102" s="1" t="s">
-        <v>258</v>
+        <v>321</v>
       </c>
       <c r="I102" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J102" s="1" t="str">
-        <f>IF(VALUE(LEFT(C102,4))&gt;2050,"Temp withdrawal",IF(F102="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C102,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="3"/>
         <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>308</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>11</v>
@@ -4515,31 +4521,31 @@
         <v>80</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>321</v>
+        <v>49</v>
       </c>
       <c r="I103" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J103" s="1" t="str">
-        <f>IF(VALUE(LEFT(C103,4))&gt;2050,"Temp withdrawal",IF(F103="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C103,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2026/27)</v>
+        <f t="shared" si="3"/>
+        <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A104" s="5" t="s">
-        <v>307</v>
+      <c r="A104" s="1" t="s">
+        <v>259</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>308</v>
+        <v>260</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>322</v>
+        <v>10</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>80</v>
@@ -4547,23 +4553,26 @@
       <c r="G104" s="1" t="s">
         <v>49</v>
       </c>
+      <c r="H104" s="1" t="s">
+        <v>261</v>
+      </c>
       <c r="I104" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J104" s="1" t="str">
-        <f>IF(VALUE(LEFT(C104,4))&gt;2050,"Temp withdrawal",IF(F104="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C104,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2027/28)</v>
+        <f t="shared" si="3"/>
+        <v>Alternates (2026/27)</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>15</v>
@@ -4575,79 +4584,49 @@
         <v>80</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>49</v>
+        <v>264</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="I105" s="1" t="s">
         <v>301</v>
       </c>
       <c r="J105" s="1" t="str">
-        <f>IF(VALUE(LEFT(C105,4))&gt;2050,"Temp withdrawal",IF(F105="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C105,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2026/27)</v>
+        <f t="shared" si="3"/>
+        <v>Alternates (2027/28)</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E106" s="1" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G106" s="1" t="s">
-        <v>264</v>
+        <v>13</v>
       </c>
       <c r="H106" s="1" t="s">
-        <v>265</v>
+        <v>170</v>
       </c>
       <c r="I106" s="1" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="J106" s="1" t="str">
-        <f>IF(VALUE(LEFT(C106,4))&gt;2050,"Temp withdrawal",IF(F106="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C106,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
-        <v>Alternates (2027/28)</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A107" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I107" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="J107" s="1" t="str">
-        <f>IF(VALUE(LEFT(C107,4))&gt;2050,"Temp withdrawal",IF(F107="No","Runs every year",IF(ISEVEN(VALUE(LEFT(C107,4))),"Alternates (2026/27)","Alternates (2027/28)")))</f>
+        <f t="shared" si="3"/>
         <v>Runs every year</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J107">
-    <sortCondition ref="A2:A107"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J106">
+    <sortCondition ref="A2:A106"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>